<commit_message>
Fix header-detection bug that dropped valid rows containing 随意契約 in reason text; re-parse all hospitals and add Kanagawa/Shizuoka region (7 hospitals)
</commit_message>
<xml_diff>
--- a/output/さいたま赤十字病院_随意契約_X線関連.xlsx
+++ b/output/さいたま赤十字病院_随意契約_X線関連.xlsx
@@ -701,7 +701,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>不明（令和7年10月6日〜令和7年10月1日）</t>
+          <t>不明（令和7年10月6日〜令和7年12月25日）</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Broaden X-ray keyword matching (portable X-ray, X-ray fluoroscopy variants, cardio-vascular X-ray) to catch real contract-name variants missed by the original keyword list; rebuild all Excel outputs
</commit_message>
<xml_diff>
--- a/output/さいたま赤十字病院_随意契約_X線関連.xlsx
+++ b/output/さいたま赤十字病院_随意契約_X線関連.xlsx
@@ -74,17 +74,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -452,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -525,6 +528,48 @@
           <t>備考</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>移動型デジタル式汎用X線透視診断装置</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>さいたま赤十字病院用度課埼玉県さいたま市中央区新都心１－５</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>令和7年5月30日</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>株式会社 栗原医療機器店 さいたま支店 さいたま市見沼区東大宮6-3-1</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>19250000</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.saitama-med.jrc.or.jp/albums/abm00003351.pdf</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>外科用イメージ（可搬型Cアーム透視装置）</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>製品</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -553,178 +598,174 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>装置カテゴリ</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>該当件数</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>一般撮影（レントゲン）</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>公表された随意契約に該当なし</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>透視撮影台（X線テレビ）</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>公表された随意契約に該当なし</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>血管撮影（CVS、アンギオ）</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>公表された随意契約に該当なし</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>外科用イメージ（可搬型Cアーム透視装置）</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>回診用X線装置</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>公表された随意契約に該当なし</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>回診用X線装置</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>公表された随意契約に該当なし</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>データソース（随意契約に関する公示 PDF）</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>対象年度</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>掲載件数</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>不明（令和7年5月29日〜令和7年5月28日）</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>https://www.saitama-med.jrc.or.jp/albums/abm00003351.pdf</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="3" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>不明（令和7年7月14日〜令和7年8月27日）</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>https://www.saitama-med.jrc.or.jp/albums/abm00003503.pdf</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="3" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>不明（令和7年10月6日〜令和7年12月25日）</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>https://www.saitama-med.jrc.or.jp/albums/abm00003576.pdf</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="3" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>不明（令和8年1月14日〜令和8年1月16日）</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>https://www.saitama-med.jrc.or.jp/albums/abm00003746.pdf</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="3" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>